<commit_message>
Implement configurable limited tournament rounds
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/niclasl/src/hockey/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9039055A-2282-B149-8CC9-87330774E072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48232ABC-9AEF-E345-AFAC-BAF09175A0D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-26240" yWindow="0" windowWidth="26240" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="83">
   <si>
     <t>age_group</t>
   </si>
@@ -269,6 +269,9 @@
   </si>
   <si>
     <t>fixed_allocation</t>
+  </si>
+  <si>
+    <t>rounds_per_tournament</t>
   </si>
 </sst>
 </file>
@@ -648,7 +651,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -656,9 +659,10 @@
     <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -677,8 +681,11 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -697,8 +704,11 @@
       <c r="F2">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -717,8 +727,11 @@
       <c r="F3">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -737,8 +750,11 @@
       <c r="F4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -757,8 +773,11 @@
       <c r="F5">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -777,8 +796,11 @@
       <c r="F6">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -797,8 +819,11 @@
       <c r="F7">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -817,8 +842,11 @@
       <c r="F8">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -837,8 +865,11 @@
       <c r="F9">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -856,6 +887,9 @@
       </c>
       <c r="F10">
         <v>5</v>
+      </c>
+      <c r="G10">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2458,8 +2492,8 @@
   <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="88.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
corrected tournament length in minutes for all groups
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/niclasl/src/hockey/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48232ABC-9AEF-E345-AFAC-BAF09175A0D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B23DEA-2879-B849-9E99-4B94A5908F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26240" yWindow="0" windowWidth="26240" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20340" yWindow="-340" windowWidth="26240" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Innstillinger" sheetId="1" r:id="rId1"/>
@@ -696,7 +696,7 @@
         <v>15</v>
       </c>
       <c r="D2">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -719,7 +719,7 @@
         <v>15</v>
       </c>
       <c r="D3">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -742,7 +742,7 @@
         <v>15</v>
       </c>
       <c r="D4">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -765,7 +765,7 @@
         <v>15</v>
       </c>
       <c r="D5">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -788,7 +788,7 @@
         <v>15</v>
       </c>
       <c r="D6">
-        <v>135</v>
+        <v>105</v>
       </c>
       <c r="E6">
         <v>4</v>
@@ -811,7 +811,7 @@
         <v>15</v>
       </c>
       <c r="D7">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="E7">
         <v>4</v>
@@ -834,7 +834,7 @@
         <v>15</v>
       </c>
       <c r="D8">
-        <v>135</v>
+        <v>105</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -880,7 +880,7 @@
         <v>15</v>
       </c>
       <c r="D10">
-        <v>175</v>
+        <v>75</v>
       </c>
       <c r="E10">
         <v>5</v>

</xml_diff>

<commit_message>
changed number of rounds
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/niclasl/src/hockey/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B23DEA-2879-B849-9E99-4B94A5908F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB773CBC-8EC5-9045-A13E-20F2FC1DEADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20340" yWindow="-340" windowWidth="26240" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="520" windowWidth="26240" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Innstillinger" sheetId="1" r:id="rId1"/>
@@ -774,7 +774,7 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
added 10minutes for each icetime to accomodate for ice preparations
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/niclasl/src/hockey/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB773CBC-8EC5-9045-A13E-20F2FC1DEADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B56CE38-B7F3-BC48-AB75-6C4414290F0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="520" windowWidth="26240" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-42560" yWindow="-1080" windowWidth="26240" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Innstillinger" sheetId="1" r:id="rId1"/>
@@ -696,7 +696,7 @@
         <v>15</v>
       </c>
       <c r="D2">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -719,7 +719,7 @@
         <v>15</v>
       </c>
       <c r="D3">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -742,7 +742,7 @@
         <v>15</v>
       </c>
       <c r="D4">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -765,7 +765,7 @@
         <v>15</v>
       </c>
       <c r="D5">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -788,7 +788,7 @@
         <v>15</v>
       </c>
       <c r="D6">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="E6">
         <v>4</v>
@@ -811,7 +811,7 @@
         <v>15</v>
       </c>
       <c r="D7">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="E7">
         <v>4</v>
@@ -834,7 +834,7 @@
         <v>15</v>
       </c>
       <c r="D8">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -857,7 +857,7 @@
         <v>15</v>
       </c>
       <c r="D9">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E9">
         <v>6</v>
@@ -880,7 +880,7 @@
         <v>15</v>
       </c>
       <c r="D10">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E10">
         <v>5</v>

</xml_diff>

<commit_message>
export and input updated icetime
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/niclasl/src/hockey/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B56CE38-B7F3-BC48-AB75-6C4414290F0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C0366A-4117-D648-A1B7-34891BC5590E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-42560" yWindow="-1080" windowWidth="26240" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,20 @@
     <sheet name="Lag" sheetId="3" r:id="rId3"/>
     <sheet name="Kilder" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -788,7 +801,7 @@
         <v>15</v>
       </c>
       <c r="D6">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E6">
         <v>4</v>
@@ -811,7 +824,7 @@
         <v>15</v>
       </c>
       <c r="D7">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E7">
         <v>4</v>
@@ -834,7 +847,7 @@
         <v>15</v>
       </c>
       <c r="D8">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -894,6 +907,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add season quality baseline (accept/advance/replace/show) with regression classification
Lets an operator accept the current non-hard finding set as a season's
regression reference so `season findings` can report KNOWN/IMPROVED/
RESOLVED/REGRESSED/NEW instead of re-listing the same accepted debt,
and wires the active baseline into canonical export evidence and the
audit context.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/niclasl/src/hockey/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C0366A-4117-D648-A1B7-34891BC5590E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F61CF061-C25C-9144-8DF0-7A8F6FFEDAB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-42560" yWindow="-1080" windowWidth="26240" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -709,7 +709,7 @@
         <v>15</v>
       </c>
       <c r="D2">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -732,7 +732,7 @@
         <v>15</v>
       </c>
       <c r="D3">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -755,7 +755,7 @@
         <v>15</v>
       </c>
       <c r="D4">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -778,7 +778,7 @@
         <v>15</v>
       </c>
       <c r="D5">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -801,7 +801,7 @@
         <v>15</v>
       </c>
       <c r="D6">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="E6">
         <v>4</v>
@@ -824,7 +824,7 @@
         <v>15</v>
       </c>
       <c r="D7">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="E7">
         <v>4</v>
@@ -847,7 +847,7 @@
         <v>15</v>
       </c>
       <c r="D8">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -870,7 +870,7 @@
         <v>15</v>
       </c>
       <c r="D9">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="E9">
         <v>6</v>
@@ -893,7 +893,7 @@
         <v>15</v>
       </c>
       <c r="D10">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="E10">
         <v>5</v>

</xml_diff>

<commit_message>
chore(season 2026-2027): checkpoint JU8 renames and accepted calendar intervals
Canonical checkpoint before publication, not a publication:

- Rename JU8 teams: Jutul Kittens -> Wildcats Rosa, Jar -> Wildcats Turkis
  (season rename-team, request rename-ju8-wildcats-2026-10-30, applied after
  the #878 fix). Placements and participant assignments unchanged.
- Eight accepted calendar booking intervals (rvv-0034, 0040, 0051, 0052,
  0077, 0090, 0165, 0179), each matching its calendar event in the
  2026-10-27 snapshot to the minute. rvv-0179 is 13:30-14:50 (80 min).
- Export directory export/2026-10-30T0912/ is not included; it is not
  published and is not part of this checkpoint.

Publication remains on hold. Stale approvals rvv-0156 and rvv-0094 are
unchanged (stale since 2026-10-01, predate the rename).

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1080,7 +1080,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">

</xml_diff>

<commit_message>
chore(season): checkpoint JU8 renames and accepted booking intervals (#879)
Canonical checkpoint only. Publication remains on hold: the two stale approvals (rvv-0156, rvv-0094) and the calendar refresh are separate steps. Nothing is published by this commit.
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1080,7 +1080,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Jar</t>
+          <t>Wildcats Turkis</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jutul Kittens</t>
+          <t>Wildcats Rosa</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">

</xml_diff>